<commit_message>
indexation de lion ratee
</commit_message>
<xml_diff>
--- a/indexation-estampes.xlsx
+++ b/indexation-estampes.xlsx
@@ -6,11 +6,11 @@
     <sheet state="visible" name="Feuille 1" sheetId="1" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName hidden="1" localSheetId="0" name="Z_9C72371F_0E2C_4FFE_8A69_38EA37B46DE5_.wvu.FilterData">'Feuille 1'!$A$1:$AC$678</definedName>
+    <definedName hidden="1" localSheetId="0" name="Z_BE891185_2BCE_4368_9F2F_D1CEAA962AFF_.wvu.FilterData">'Feuille 1'!$A$1:$AC$678</definedName>
   </definedNames>
   <calcPr/>
   <customWorkbookViews>
-    <customWorkbookView activeSheetId="0" maximized="1" windowHeight="0" windowWidth="0" guid="{9C72371F-0E2C-4FFE-8A69-38EA37B46DE5}" name="Filtre 1"/>
+    <customWorkbookView activeSheetId="0" maximized="1" windowHeight="0" windowWidth="0" guid="{BE891185-2BCE-4368-9F2F-D1CEAA962AFF}" name="Filtre 1"/>
   </customWorkbookViews>
 </workbook>
 </file>
@@ -5011,7 +5011,7 @@
     <t>emblématique ; personnification des vices et des vertus ; héraldique ; mythologie gréco-romaine ; personnification des villes, des États et des fleuves ; personnification</t>
   </si>
   <si>
-    <t>temple ; soleil ; armoiries ; Renommée (personnification) ; Victoire (personnification) ; lion (animal) ; pyramide ; amours ; corne d'abondance ; globe terrestre ; bouclier ; massue ; rameau d'olivier ; France (personnification) ; trophée ; Bavière (personnification) ; Hymen (personnification) ; Paix (personnification) ; Valeur (personnification) ; lion ; palme ;</t>
+    <t>temple ; soleil ; armoiries ; Renommée (personnification) ; Victoire (personnification) ; lion (animal) ; pyramide ; amours ; corne d'abondance ; globe terrestre ; bouclier ; massue ; rameau d'olivier ; France (personnification) ; trophée ; Bavière (personnification) ; Hymen (personnification) ; Paix (personnification) ; Valeur (personnification) ; lion (animal) ; palme ;</t>
   </si>
   <si>
     <r>
@@ -27951,7 +27951,7 @@
       <c r="M131" s="36" t="s">
         <v>1213</v>
       </c>
-      <c r="N131" s="38" t="s">
+      <c r="N131" s="179" t="s">
         <v>1214</v>
       </c>
       <c r="O131" s="38"/>
@@ -62767,7 +62767,7 @@
     </row>
   </sheetData>
   <customSheetViews>
-    <customSheetView guid="{9C72371F-0E2C-4FFE-8A69-38EA37B46DE5}" filter="1" showAutoFilter="1">
+    <customSheetView guid="{BE891185-2BCE-4368-9F2F-D1CEAA962AFF}" filter="1" showAutoFilter="1">
       <autoFilter ref="$A$1:$AC$678"/>
     </customSheetView>
   </customSheetViews>

</xml_diff>

<commit_message>
fix wrong  opentheso id lieu associe
</commit_message>
<xml_diff>
--- a/indexation-estampes.xlsx
+++ b/indexation-estampes.xlsx
@@ -6,11 +6,11 @@
     <sheet state="visible" name="Feuille 1" sheetId="1" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName hidden="1" localSheetId="0" name="Z_7D2142DF_EA57_49EF_9659_14F3963649E6_.wvu.FilterData">'Feuille 1'!$A$1:$AC$678</definedName>
+    <definedName hidden="1" localSheetId="0" name="Z_65CD057B_49E3_482E_A40A_F23D7F7626AA_.wvu.FilterData">'Feuille 1'!$A$1:$AC$678</definedName>
   </definedNames>
   <calcPr/>
   <customWorkbookViews>
-    <customWorkbookView activeSheetId="0" maximized="1" windowHeight="0" windowWidth="0" guid="{7D2142DF-EA57-49EF-9659-14F3963649E6}" name="Filtre 1"/>
+    <customWorkbookView activeSheetId="0" maximized="1" windowHeight="0" windowWidth="0" guid="{65CD057B-49E3-482E-A40A-F23D7F7626AA}" name="Filtre 1"/>
   </customWorkbookViews>
 </workbook>
 </file>
@@ -16046,7 +16046,7 @@
     <t>[Jetons de l'année 1703]*</t>
   </si>
   <si>
-    <t>MEUDON : 2911</t>
+    <t xml:space="preserve">2911: MEUDON </t>
   </si>
   <si>
     <t>emblématique ; personnification des villes, des États et des fleuves ; mythologie gréco-romaine ; architecture</t>
@@ -52676,7 +52676,7 @@
       </c>
       <c r="J464" s="106"/>
       <c r="K464" s="22"/>
-      <c r="L464" s="22" t="s">
+      <c r="L464" s="192" t="s">
         <v>3859</v>
       </c>
       <c r="M464" s="169" t="s">
@@ -62767,7 +62767,7 @@
     </row>
   </sheetData>
   <customSheetViews>
-    <customSheetView guid="{7D2142DF-EA57-49EF-9659-14F3963649E6}" filter="1" showAutoFilter="1">
+    <customSheetView guid="{65CD057B-49E3-482E-A40A-F23D7F7626AA}" filter="1" showAutoFilter="1">
       <autoFilter ref="$A$1:$AC$678"/>
     </customSheetView>
   </customSheetViews>

</xml_diff>